<commit_message>
Pine Island Plaza: update proforma to 4.5% 30-Yr Am seller carry, 50K capex, new rent roll & financials
</commit_message>
<xml_diff>
--- a/pine-island-plaza/files/Pine-Island-Plaza-Proforma.xlsx
+++ b/pine-island-plaza/files/Pine-Island-Plaza-Proforma.xlsx
@@ -11,14 +11,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="tB9oyjFSot/RGCjU/YVnNgDt8dqszQepvDct68ykdNM="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="eCFgHEPlAVBpWBvOMDxrytjLHwqrukHKomEKFXeqwHE="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="118">
   <si>
     <t>Location</t>
   </si>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>Terms</t>
-  </si>
-  <si>
-    <t>I/O</t>
   </si>
   <si>
     <t>INCOME</t>
@@ -197,13 +194,13 @@
     <t>7% Cap Rate</t>
   </si>
   <si>
+    <t>6.5% Cap Rate</t>
+  </si>
+  <si>
     <t>6% Cap Rate</t>
   </si>
   <si>
-    <t>5% Cap Rate</t>
-  </si>
-  <si>
-    <t>4% Cap Rate</t>
+    <t>5.5% Cap Rate</t>
   </si>
   <si>
     <t>CAM</t>
@@ -751,7 +748,7 @@
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
+      <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="bottom"/>
@@ -928,7 +925,7 @@
     <xf borderId="17" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="18" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="11" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="top"/>
+      <alignment readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" vertical="top"/>
@@ -969,7 +966,7 @@
     </xf>
     <xf borderId="11" fillId="6" fontId="21" numFmtId="165" xfId="0" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="19" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="19" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -1559,11 +1556,11 @@
         <v>10</v>
       </c>
       <c r="D11" s="11">
-        <v>342000.0</v>
+        <v>250000.0</v>
       </c>
       <c r="E11" s="14">
         <f>D11/D6</f>
-        <v>0.1005882353</v>
+        <v>0.07352941176</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1596,7 +1593,7 @@
       </c>
       <c r="D12" s="13">
         <f>SUM(D8:D11)</f>
-        <v>1650000</v>
+        <v>1558000</v>
       </c>
       <c r="E12" s="14">
         <f>E6+E9</f>
@@ -1632,7 +1629,7 @@
         <v>12</v>
       </c>
       <c r="D13" s="15">
-        <v>0.055</v>
+        <v>0.045</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -1664,8 +1661,8 @@
       <c r="C14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="16" t="s">
-        <v>14</v>
+      <c r="D14" s="16">
+        <v>30.0</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
@@ -1753,38 +1750,38 @@
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="18" t="s">
+      <c r="G17" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="19" t="s">
+      <c r="H17" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="19" t="s">
+      <c r="I17" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="19" t="s">
+      <c r="J17" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="J17" s="19" t="s">
+      <c r="K17" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="K17" s="19" t="s">
+      <c r="L17" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="L17" s="19" t="s">
+      <c r="M17" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="M17" s="19" t="s">
+      <c r="N17" s="19" t="s">
         <v>24</v>
-      </c>
-      <c r="N17" s="19" t="s">
-        <v>25</v>
       </c>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
@@ -1833,48 +1830,48 @@
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D19" s="21"/>
       <c r="E19" s="22">
         <f>'7 YR - Rent Roll'!F17</f>
-        <v>265112</v>
+        <v>265612</v>
       </c>
       <c r="F19" s="22">
         <f>'7 YR - Rent Roll'!G17</f>
-        <v>271729.5</v>
+        <v>277275</v>
       </c>
       <c r="G19" s="22">
         <f>'7 YR - Rent Roll'!H17</f>
-        <v>285315.975</v>
+        <v>291138.75</v>
       </c>
       <c r="H19" s="23">
         <f>'7 YR - Rent Roll'!I17</f>
-        <v>299581.7738</v>
+        <v>305695.6875</v>
       </c>
       <c r="I19" s="22">
         <f>'7 YR - Rent Roll'!J17</f>
-        <v>314560.8624</v>
+        <v>320980.4719</v>
       </c>
       <c r="J19" s="22">
         <f>'7 YR - Rent Roll'!K17</f>
-        <v>330288.9056</v>
+        <v>337029.4955</v>
       </c>
       <c r="K19" s="22">
         <f>'7 YR - Rent Roll'!L17</f>
-        <v>346803.3508</v>
+        <v>353880.9702</v>
       </c>
       <c r="L19" s="22">
         <f>'7 YR - Rent Roll'!M17</f>
-        <v>364143.5184</v>
+        <v>371575.0188</v>
       </c>
       <c r="M19" s="22">
         <f>'7 YR - Rent Roll'!N17</f>
-        <v>382350.6943</v>
+        <v>390153.7697</v>
       </c>
       <c r="N19" s="22">
         <f>'7 YR - Rent Roll'!O17</f>
-        <v>401468.229</v>
+        <v>409661.4582</v>
       </c>
       <c r="O19" s="22" t="str">
         <f>'7 YR - Rent Roll'!P17</f>
@@ -1900,7 +1897,7 @@
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D20" s="21"/>
       <c r="E20" s="24">
@@ -1988,48 +1985,48 @@
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D22" s="28"/>
       <c r="E22" s="29">
         <f t="shared" ref="E22:N22" si="2">SUM(E19:E20)</f>
-        <v>313361.17</v>
+        <v>313861.17</v>
       </c>
       <c r="F22" s="29">
         <f t="shared" si="2"/>
-        <v>389729.5</v>
+        <v>395275</v>
       </c>
       <c r="G22" s="29">
         <f t="shared" si="2"/>
-        <v>407315.975</v>
+        <v>413138.75</v>
       </c>
       <c r="H22" s="29">
         <f t="shared" si="2"/>
-        <v>425241.7738</v>
+        <v>431355.6875</v>
       </c>
       <c r="I22" s="29">
         <f t="shared" si="2"/>
-        <v>443990.6624</v>
+        <v>450410.2719</v>
       </c>
       <c r="J22" s="29">
         <f t="shared" si="2"/>
-        <v>463601.5996</v>
+        <v>470342.1895</v>
       </c>
       <c r="K22" s="29">
         <f t="shared" si="2"/>
-        <v>484115.4257</v>
+        <v>491193.0451</v>
       </c>
       <c r="L22" s="29">
         <f t="shared" si="2"/>
-        <v>505574.9554</v>
+        <v>513006.4558</v>
       </c>
       <c r="M22" s="29">
         <f t="shared" si="2"/>
-        <v>528025.0745</v>
+        <v>535828.1499</v>
       </c>
       <c r="N22" s="29">
         <f t="shared" si="2"/>
-        <v>551512.8406</v>
+        <v>559706.0698</v>
       </c>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
@@ -2078,7 +2075,7 @@
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D24" s="31">
         <v>0.05</v>
@@ -2088,39 +2085,39 @@
       </c>
       <c r="F24" s="32">
         <f t="shared" ref="F24:N24" si="3">F22*$D$24*-1</f>
-        <v>-19486.475</v>
+        <v>-19763.75</v>
       </c>
       <c r="G24" s="32">
         <f t="shared" si="3"/>
-        <v>-20365.79875</v>
+        <v>-20656.9375</v>
       </c>
       <c r="H24" s="32">
         <f t="shared" si="3"/>
-        <v>-21262.08869</v>
+        <v>-21567.78438</v>
       </c>
       <c r="I24" s="32">
         <f t="shared" si="3"/>
-        <v>-22199.53312</v>
+        <v>-22520.51359</v>
       </c>
       <c r="J24" s="32">
         <f t="shared" si="3"/>
-        <v>-23180.07998</v>
+        <v>-23517.10947</v>
       </c>
       <c r="K24" s="32">
         <f t="shared" si="3"/>
-        <v>-24205.77128</v>
+        <v>-24559.65225</v>
       </c>
       <c r="L24" s="32">
         <f t="shared" si="3"/>
-        <v>-25278.74777</v>
+        <v>-25650.32279</v>
       </c>
       <c r="M24" s="32">
         <f t="shared" si="3"/>
-        <v>-26401.25372</v>
+        <v>-26791.40749</v>
       </c>
       <c r="N24" s="32">
         <f t="shared" si="3"/>
-        <v>-27575.64203</v>
+        <v>-27985.30349</v>
       </c>
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
@@ -2169,48 +2166,48 @@
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D26" s="33"/>
       <c r="E26" s="29">
         <f t="shared" ref="E26:N26" si="4">E22+E24</f>
-        <v>313361.17</v>
+        <v>313861.17</v>
       </c>
       <c r="F26" s="29">
         <f t="shared" si="4"/>
-        <v>370243.025</v>
+        <v>375511.25</v>
       </c>
       <c r="G26" s="29">
         <f t="shared" si="4"/>
-        <v>386950.1763</v>
+        <v>392481.8125</v>
       </c>
       <c r="H26" s="29">
         <f t="shared" si="4"/>
-        <v>403979.6851</v>
+        <v>409787.9031</v>
       </c>
       <c r="I26" s="29">
         <f t="shared" si="4"/>
-        <v>421791.1293</v>
+        <v>427889.7583</v>
       </c>
       <c r="J26" s="29">
         <f t="shared" si="4"/>
-        <v>440421.5196</v>
+        <v>446825.08</v>
       </c>
       <c r="K26" s="29">
         <f t="shared" si="4"/>
-        <v>459909.6544</v>
+        <v>466633.3928</v>
       </c>
       <c r="L26" s="29">
         <f t="shared" si="4"/>
-        <v>480296.2077</v>
+        <v>487356.133</v>
       </c>
       <c r="M26" s="29">
         <f t="shared" si="4"/>
-        <v>501623.8208</v>
+        <v>509036.7424</v>
       </c>
       <c r="N26" s="29">
         <f t="shared" si="4"/>
-        <v>523937.1986</v>
+        <v>531720.7663</v>
       </c>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
@@ -2259,7 +2256,7 @@
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -2319,7 +2316,7 @@
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="34">
@@ -2370,7 +2367,7 @@
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="34">
@@ -2421,48 +2418,48 @@
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="35" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="34">
         <f>E26*0.05</f>
-        <v>15668.0585</v>
+        <v>15693.0585</v>
       </c>
       <c r="F32" s="34">
         <f t="shared" ref="F32:N32" si="5">F26*0.06</f>
-        <v>22214.5815</v>
+        <v>22530.675</v>
       </c>
       <c r="G32" s="34">
         <f t="shared" si="5"/>
-        <v>23217.01058</v>
+        <v>23548.90875</v>
       </c>
       <c r="H32" s="34">
         <f t="shared" si="5"/>
-        <v>24238.7811</v>
+        <v>24587.27419</v>
       </c>
       <c r="I32" s="34">
         <f t="shared" si="5"/>
-        <v>25307.46776</v>
+        <v>25673.3855</v>
       </c>
       <c r="J32" s="34">
         <f t="shared" si="5"/>
-        <v>26425.29117</v>
+        <v>26809.5048</v>
       </c>
       <c r="K32" s="34">
         <f t="shared" si="5"/>
-        <v>27594.57926</v>
+        <v>27998.00357</v>
       </c>
       <c r="L32" s="34">
         <f t="shared" si="5"/>
-        <v>28817.77246</v>
+        <v>29241.36798</v>
       </c>
       <c r="M32" s="34">
         <f t="shared" si="5"/>
-        <v>30097.42925</v>
+        <v>30542.20454</v>
       </c>
       <c r="N32" s="34">
         <f t="shared" si="5"/>
-        <v>31436.23191</v>
+        <v>31903.24598</v>
       </c>
       <c r="O32" s="1"/>
       <c r="P32" s="1"/>
@@ -2482,7 +2479,7 @@
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="36">
@@ -2490,39 +2487,39 @@
       </c>
       <c r="F33" s="34">
         <f t="shared" ref="F33:N33" si="6">F26*0.02</f>
-        <v>7404.8605</v>
+        <v>7510.225</v>
       </c>
       <c r="G33" s="34">
         <f t="shared" si="6"/>
-        <v>7739.003525</v>
+        <v>7849.63625</v>
       </c>
       <c r="H33" s="34">
         <f t="shared" si="6"/>
-        <v>8079.593701</v>
+        <v>8195.758063</v>
       </c>
       <c r="I33" s="34">
         <f t="shared" si="6"/>
-        <v>8435.822586</v>
+        <v>8557.795166</v>
       </c>
       <c r="J33" s="34">
         <f t="shared" si="6"/>
-        <v>8808.430392</v>
+        <v>8936.5016</v>
       </c>
       <c r="K33" s="34">
         <f t="shared" si="6"/>
-        <v>9198.193087</v>
+        <v>9332.667856</v>
       </c>
       <c r="L33" s="34">
         <f t="shared" si="6"/>
-        <v>9605.924153</v>
+        <v>9747.122661</v>
       </c>
       <c r="M33" s="34">
         <f t="shared" si="6"/>
-        <v>10032.47642</v>
+        <v>10180.73485</v>
       </c>
       <c r="N33" s="34">
         <f t="shared" si="6"/>
-        <v>10478.74397</v>
+        <v>10634.41533</v>
       </c>
       <c r="O33" s="1"/>
       <c r="P33" s="1"/>
@@ -2542,7 +2539,7 @@
       <c r="A34" s="37"/>
       <c r="B34" s="1"/>
       <c r="C34" s="20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="38">
@@ -2602,7 +2599,7 @@
       <c r="A35" s="40"/>
       <c r="B35" s="40"/>
       <c r="C35" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="39">
@@ -2663,7 +2660,7 @@
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="34">
@@ -2714,7 +2711,7 @@
       <c r="A37" s="40"/>
       <c r="B37" s="1"/>
       <c r="C37" s="35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="34">
@@ -2774,7 +2771,7 @@
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="34">
@@ -2834,7 +2831,7 @@
       <c r="A39" s="40"/>
       <c r="B39" s="1"/>
       <c r="C39" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="34">
@@ -2894,7 +2891,7 @@
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="34"/>
@@ -2980,48 +2977,48 @@
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D42" s="41"/>
       <c r="E42" s="29">
         <f t="shared" ref="E42:N42" si="13">SUM(E30:E40)</f>
-        <v>88383.6585</v>
+        <v>88408.6585</v>
       </c>
       <c r="F42" s="29">
         <f t="shared" si="13"/>
-        <v>120115.51</v>
+        <v>120536.968</v>
       </c>
       <c r="G42" s="29">
         <f t="shared" si="13"/>
-        <v>124085.9641</v>
+        <v>124528.495</v>
       </c>
       <c r="H42" s="29">
         <f t="shared" si="13"/>
-        <v>128161.2233</v>
+        <v>128625.8808</v>
       </c>
       <c r="I42" s="29">
         <f t="shared" si="13"/>
-        <v>132380.4243</v>
+        <v>132868.3147</v>
       </c>
       <c r="J42" s="29">
         <f t="shared" si="13"/>
-        <v>136748.9696</v>
+        <v>137261.2544</v>
       </c>
       <c r="K42" s="29">
         <f t="shared" si="13"/>
-        <v>141272.4778</v>
+        <v>141810.3769</v>
       </c>
       <c r="L42" s="29">
         <f t="shared" si="13"/>
-        <v>145956.7932</v>
+        <v>146521.5873</v>
       </c>
       <c r="M42" s="29">
         <f t="shared" si="13"/>
-        <v>150807.9952</v>
+        <v>151401.0289</v>
       </c>
       <c r="N42" s="29">
         <f t="shared" si="13"/>
-        <v>155832.4081</v>
+        <v>156455.0935</v>
       </c>
       <c r="O42" s="1"/>
       <c r="P42" s="1"/>
@@ -3070,48 +3067,48 @@
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D44" s="33"/>
       <c r="E44" s="43">
         <f t="shared" ref="E44:N44" si="14">E26-E42</f>
-        <v>224977.5115</v>
+        <v>225452.5115</v>
       </c>
       <c r="F44" s="43">
         <f t="shared" si="14"/>
-        <v>250127.515</v>
+        <v>254974.282</v>
       </c>
       <c r="G44" s="43">
         <f t="shared" si="14"/>
-        <v>262864.2121</v>
+        <v>267953.3175</v>
       </c>
       <c r="H44" s="43">
         <f t="shared" si="14"/>
-        <v>275818.4617</v>
+        <v>281162.0223</v>
       </c>
       <c r="I44" s="43">
         <f t="shared" si="14"/>
-        <v>289410.705</v>
+        <v>295021.4436</v>
       </c>
       <c r="J44" s="43">
         <f t="shared" si="14"/>
-        <v>303672.55</v>
+        <v>309563.8256</v>
       </c>
       <c r="K44" s="43">
         <f t="shared" si="14"/>
-        <v>318637.1766</v>
+        <v>324823.0159</v>
       </c>
       <c r="L44" s="43">
         <f t="shared" si="14"/>
-        <v>334339.4144</v>
+        <v>340834.5458</v>
       </c>
       <c r="M44" s="43">
         <f t="shared" si="14"/>
-        <v>350815.8256</v>
+        <v>357635.7135</v>
       </c>
       <c r="N44" s="43">
         <f t="shared" si="14"/>
-        <v>368104.7905</v>
+        <v>375265.6728</v>
       </c>
       <c r="O44" s="1"/>
       <c r="P44" s="1"/>
@@ -3160,48 +3157,48 @@
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="45">
-        <f t="shared" ref="E46:N46" si="15">-$D$13*$D$7</f>
-        <v>-121000</v>
+        <f>PMT(D13, D14, D7, 0)</f>
+        <v>-135061.3944</v>
       </c>
       <c r="F46" s="45">
-        <f t="shared" si="15"/>
-        <v>-121000</v>
+        <f t="shared" ref="F46:K46" si="15">E46</f>
+        <v>-135061.3944</v>
       </c>
       <c r="G46" s="45">
         <f t="shared" si="15"/>
-        <v>-121000</v>
+        <v>-135061.3944</v>
       </c>
       <c r="H46" s="45">
         <f t="shared" si="15"/>
-        <v>-121000</v>
+        <v>-135061.3944</v>
       </c>
       <c r="I46" s="45">
         <f t="shared" si="15"/>
-        <v>-121000</v>
+        <v>-135061.3944</v>
       </c>
       <c r="J46" s="45">
         <f t="shared" si="15"/>
-        <v>-121000</v>
+        <v>-135061.3944</v>
       </c>
       <c r="K46" s="45">
         <f t="shared" si="15"/>
-        <v>-121000</v>
+        <v>-135061.3944</v>
       </c>
       <c r="L46" s="45">
-        <f t="shared" si="15"/>
-        <v>-121000</v>
+        <f t="shared" ref="L46:N46" si="16">-$D$13*$D$7</f>
+        <v>-99000</v>
       </c>
       <c r="M46" s="45">
-        <f t="shared" si="15"/>
-        <v>-121000</v>
+        <f t="shared" si="16"/>
+        <v>-99000</v>
       </c>
       <c r="N46" s="45">
-        <f t="shared" si="15"/>
-        <v>-121000</v>
+        <f t="shared" si="16"/>
+        <v>-99000</v>
       </c>
       <c r="O46" s="1"/>
       <c r="P46" s="1"/>
@@ -3250,48 +3247,48 @@
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D48" s="48"/>
       <c r="E48" s="49">
-        <f t="shared" ref="E48:N48" si="16">SUM(E44:E46)</f>
-        <v>103977.5115</v>
+        <f t="shared" ref="E48:N48" si="17">SUM(E44:E46)</f>
+        <v>90391.1171</v>
       </c>
       <c r="F48" s="49">
-        <f t="shared" si="16"/>
-        <v>129127.515</v>
+        <f t="shared" si="17"/>
+        <v>119912.8876</v>
       </c>
       <c r="G48" s="49">
-        <f t="shared" si="16"/>
-        <v>141864.2121</v>
+        <f t="shared" si="17"/>
+        <v>132891.9231</v>
       </c>
       <c r="H48" s="49">
-        <f t="shared" si="16"/>
-        <v>154818.4617</v>
+        <f t="shared" si="17"/>
+        <v>146100.6279</v>
       </c>
       <c r="I48" s="49">
-        <f t="shared" si="16"/>
-        <v>168410.705</v>
+        <f t="shared" si="17"/>
+        <v>159960.0492</v>
       </c>
       <c r="J48" s="49">
-        <f t="shared" si="16"/>
-        <v>182672.55</v>
+        <f t="shared" si="17"/>
+        <v>174502.4312</v>
       </c>
       <c r="K48" s="49">
-        <f t="shared" si="16"/>
-        <v>197637.1766</v>
+        <f t="shared" si="17"/>
+        <v>189761.6215</v>
       </c>
       <c r="L48" s="49">
-        <f t="shared" si="16"/>
-        <v>213339.4144</v>
+        <f t="shared" si="17"/>
+        <v>241834.5458</v>
       </c>
       <c r="M48" s="49">
-        <f t="shared" si="16"/>
-        <v>229815.8256</v>
+        <f t="shared" si="17"/>
+        <v>258635.7135</v>
       </c>
       <c r="N48" s="49">
-        <f t="shared" si="16"/>
-        <v>247104.7905</v>
+        <f t="shared" si="17"/>
+        <v>276265.6728</v>
       </c>
       <c r="O48" s="1"/>
       <c r="P48" s="1"/>
@@ -3340,48 +3337,48 @@
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="51" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D50" s="52"/>
       <c r="E50" s="53">
         <f>E44/(D6+D9)</f>
-        <v>0.06540043939</v>
+        <v>0.06553852078</v>
       </c>
       <c r="F50" s="53">
-        <f t="shared" ref="F50:N50" si="17">F44/($D$6+$D$9)</f>
-        <v>0.07271148692</v>
+        <f t="shared" ref="F50:N50" si="18">F44/($D$6+$D$9)</f>
+        <v>0.07412043081</v>
       </c>
       <c r="G50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.07641401515</v>
+        <f t="shared" si="18"/>
+        <v>0.07789340624</v>
       </c>
       <c r="H50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.08017978538</v>
+        <f t="shared" si="18"/>
+        <v>0.08173314603</v>
       </c>
       <c r="I50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.08413101889</v>
+        <f t="shared" si="18"/>
+        <v>0.08576204756</v>
       </c>
       <c r="J50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.08827690407</v>
+        <f t="shared" si="18"/>
+        <v>0.08998948418</v>
       </c>
       <c r="K50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.09262708621</v>
+        <f t="shared" si="18"/>
+        <v>0.09442529533</v>
       </c>
       <c r="L50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.09719169024</v>
+        <f t="shared" si="18"/>
+        <v>0.09907980982</v>
       </c>
       <c r="M50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.1019813446</v>
+        <f t="shared" si="18"/>
+        <v>0.1039638702</v>
       </c>
       <c r="N50" s="53">
-        <f t="shared" si="17"/>
-        <v>0.1070072065</v>
+        <f t="shared" si="18"/>
+        <v>0.1090888584</v>
       </c>
       <c r="O50" s="1"/>
       <c r="P50" s="1"/>
@@ -3401,48 +3398,48 @@
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="54" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="55">
-        <f t="shared" ref="E51:N51" si="18">E48/($D$12)</f>
-        <v>0.06301667364</v>
+        <f t="shared" ref="E51:N51" si="19">E48/($D$12)</f>
+        <v>0.05801740507</v>
       </c>
       <c r="F51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.0782591</v>
+        <f t="shared" si="19"/>
+        <v>0.07696590989</v>
       </c>
       <c r="G51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.08597831037</v>
+        <f t="shared" si="19"/>
+        <v>0.08529648463</v>
       </c>
       <c r="H51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.09382937074</v>
+        <f t="shared" si="19"/>
+        <v>0.09377447236</v>
       </c>
       <c r="I51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.1020670939</v>
+        <f t="shared" si="19"/>
+        <v>0.1026701215</v>
       </c>
       <c r="J51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.1107106364</v>
+        <f t="shared" si="19"/>
+        <v>0.1120041278</v>
       </c>
       <c r="K51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.119780107</v>
+        <f t="shared" si="19"/>
+        <v>0.1217982166</v>
       </c>
       <c r="L51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.1292966148</v>
+        <f t="shared" si="19"/>
+        <v>0.1552211462</v>
       </c>
       <c r="M51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.1392823185</v>
+        <f t="shared" si="19"/>
+        <v>0.1660049509</v>
       </c>
       <c r="N51" s="55">
-        <f t="shared" si="18"/>
-        <v>0.1497604791</v>
+        <f t="shared" si="19"/>
+        <v>0.1773207142</v>
       </c>
       <c r="O51" s="1"/>
       <c r="P51" s="1"/>
@@ -3462,48 +3459,48 @@
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="56" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D52" s="57"/>
       <c r="E52" s="58">
-        <f t="shared" ref="E52:N52" si="19">-E44/E46</f>
-        <v>1.859318277</v>
+        <f t="shared" ref="E52:N52" si="20">-E44/E46</f>
+        <v>1.669259469</v>
       </c>
       <c r="F52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.067169545</v>
+        <f t="shared" si="20"/>
+        <v>1.887839846</v>
       </c>
       <c r="G52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.172431505</v>
+        <f t="shared" si="20"/>
+        <v>1.983937147</v>
       </c>
       <c r="H52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.279491419</v>
+        <f t="shared" si="20"/>
+        <v>2.081734929</v>
       </c>
       <c r="I52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.391824008</v>
+        <f t="shared" si="20"/>
+        <v>2.184350642</v>
       </c>
       <c r="J52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.509690496</v>
+        <f t="shared" si="20"/>
+        <v>2.292023024</v>
       </c>
       <c r="K52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.633365096</v>
+        <f t="shared" si="20"/>
+        <v>2.405002683</v>
       </c>
       <c r="L52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.763135656</v>
+        <f t="shared" si="20"/>
+        <v>3.44277319</v>
       </c>
       <c r="M52" s="58">
-        <f t="shared" si="19"/>
-        <v>2.899304344</v>
+        <f t="shared" si="20"/>
+        <v>3.612481954</v>
       </c>
       <c r="N52" s="58">
-        <f t="shared" si="19"/>
-        <v>3.042188351</v>
+        <f t="shared" si="20"/>
+        <v>3.790562351</v>
       </c>
       <c r="O52" s="1"/>
       <c r="P52" s="1"/>
@@ -3552,23 +3549,23 @@
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="59" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D54" s="60">
         <f>-D12</f>
-        <v>-1650000</v>
+        <v>-1558000</v>
       </c>
       <c r="E54" s="61">
-        <f t="shared" ref="E54:G54" si="20">E48</f>
-        <v>103977.5115</v>
+        <f t="shared" ref="E54:G54" si="21">E48</f>
+        <v>90391.1171</v>
       </c>
       <c r="F54" s="61">
-        <f t="shared" si="20"/>
-        <v>129127.515</v>
+        <f t="shared" si="21"/>
+        <v>119912.8876</v>
       </c>
       <c r="G54" s="62">
-        <f t="shared" si="20"/>
-        <v>141864.2121</v>
+        <f t="shared" si="21"/>
+        <v>132891.9231</v>
       </c>
       <c r="H54" s="63">
         <f>115500+9502</f>
@@ -3576,27 +3573,27 @@
       </c>
       <c r="I54" s="62">
         <f>(D12*0.07)</f>
-        <v>115500</v>
+        <v>109060</v>
       </c>
       <c r="J54" s="61">
         <f>(D12*0.07)</f>
-        <v>115500</v>
+        <v>109060</v>
       </c>
       <c r="K54" s="61">
-        <f t="shared" ref="K54:N54" si="21">($D$12*0.07)</f>
-        <v>115500</v>
+        <f t="shared" ref="K54:N54" si="22">($D$12*0.07)</f>
+        <v>109060</v>
       </c>
       <c r="L54" s="61">
-        <f t="shared" si="21"/>
-        <v>115500</v>
+        <f t="shared" si="22"/>
+        <v>109060</v>
       </c>
       <c r="M54" s="61">
-        <f t="shared" si="21"/>
-        <v>115500</v>
+        <f t="shared" si="22"/>
+        <v>109060</v>
       </c>
       <c r="N54" s="61">
-        <f t="shared" si="21"/>
-        <v>115500</v>
+        <f t="shared" si="22"/>
+        <v>109060</v>
       </c>
       <c r="O54" s="1"/>
       <c r="P54" s="1"/>
@@ -3616,47 +3613,47 @@
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="59" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D55" s="64"/>
       <c r="E55" s="61">
         <v>0.0</v>
       </c>
       <c r="F55" s="61">
-        <f t="shared" ref="F55:N55" si="22">(F48-F54)/2</f>
+        <f t="shared" ref="F55:N55" si="23">(F48-F54)/2</f>
         <v>0</v>
       </c>
       <c r="G55" s="61">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="H55" s="61">
-        <f t="shared" si="22"/>
-        <v>14908.23086</v>
+        <f t="shared" si="23"/>
+        <v>10549.31397</v>
       </c>
       <c r="I55" s="61">
-        <f t="shared" si="22"/>
-        <v>26455.35249</v>
+        <f t="shared" si="23"/>
+        <v>25450.02461</v>
       </c>
       <c r="J55" s="61">
-        <f t="shared" si="22"/>
-        <v>33586.275</v>
+        <f t="shared" si="23"/>
+        <v>32721.21559</v>
       </c>
       <c r="K55" s="61">
-        <f t="shared" si="22"/>
-        <v>41068.58828</v>
+        <f t="shared" si="23"/>
+        <v>40350.81076</v>
       </c>
       <c r="L55" s="61">
-        <f t="shared" si="22"/>
-        <v>48919.70722</v>
+        <f t="shared" si="23"/>
+        <v>66387.27288</v>
       </c>
       <c r="M55" s="61">
-        <f t="shared" si="22"/>
-        <v>57157.91279</v>
+        <f t="shared" si="23"/>
+        <v>74787.85673</v>
       </c>
       <c r="N55" s="61">
-        <f t="shared" si="22"/>
-        <v>65802.39524</v>
+        <f t="shared" si="23"/>
+        <v>83602.83638</v>
       </c>
       <c r="O55" s="1"/>
       <c r="P55" s="1"/>
@@ -3676,7 +3673,7 @@
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="59" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D56" s="64"/>
       <c r="E56" s="61">
@@ -3687,36 +3684,36 @@
         <v>0</v>
       </c>
       <c r="G56" s="61">
-        <f t="shared" ref="G56:H56" si="23">G55</f>
+        <f t="shared" ref="G56:H56" si="24">G55</f>
         <v>0</v>
       </c>
       <c r="H56" s="61">
-        <f t="shared" si="23"/>
-        <v>14908.23086</v>
+        <f t="shared" si="24"/>
+        <v>10549.31397</v>
       </c>
       <c r="I56" s="61">
-        <f t="shared" ref="I56:N56" si="24">(I48-I54)/2</f>
-        <v>26455.35249</v>
+        <f t="shared" ref="I56:N56" si="25">(I48-I54)/2</f>
+        <v>25450.02461</v>
       </c>
       <c r="J56" s="61">
-        <f t="shared" si="24"/>
-        <v>33586.275</v>
+        <f t="shared" si="25"/>
+        <v>32721.21559</v>
       </c>
       <c r="K56" s="61">
-        <f t="shared" si="24"/>
-        <v>41068.58828</v>
+        <f t="shared" si="25"/>
+        <v>40350.81076</v>
       </c>
       <c r="L56" s="61">
-        <f t="shared" si="24"/>
-        <v>48919.70722</v>
+        <f t="shared" si="25"/>
+        <v>66387.27288</v>
       </c>
       <c r="M56" s="61">
-        <f t="shared" si="24"/>
-        <v>57157.91279</v>
+        <f t="shared" si="25"/>
+        <v>74787.85673</v>
       </c>
       <c r="N56" s="61">
-        <f t="shared" si="24"/>
-        <v>65802.39524</v>
+        <f t="shared" si="25"/>
+        <v>83602.83638</v>
       </c>
       <c r="O56" s="1"/>
       <c r="P56" s="1"/>
@@ -3736,48 +3733,48 @@
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="59" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D57" s="64"/>
       <c r="E57" s="65">
         <f>E54/D12</f>
-        <v>0.06301667364</v>
+        <v>0.05801740507</v>
       </c>
       <c r="F57" s="65">
         <f>(F54+F55)/D12</f>
-        <v>0.0782591</v>
+        <v>0.07696590989</v>
       </c>
       <c r="G57" s="65">
-        <f t="shared" ref="G57:N57" si="25">(G54+G55)/$D$12</f>
-        <v>0.08597831037</v>
+        <f t="shared" ref="G57:N57" si="26">(G54+G55)/$D$12</f>
+        <v>0.08529648463</v>
       </c>
       <c r="H57" s="65">
-        <f t="shared" si="25"/>
-        <v>0.08479407931</v>
+        <f t="shared" si="26"/>
+        <v>0.08700341076</v>
       </c>
       <c r="I57" s="65">
-        <f t="shared" si="25"/>
-        <v>0.08603354696</v>
+        <f t="shared" si="26"/>
+        <v>0.08633506073</v>
       </c>
       <c r="J57" s="65">
-        <f t="shared" si="25"/>
-        <v>0.09035531818</v>
+        <f t="shared" si="26"/>
+        <v>0.09100206392</v>
       </c>
       <c r="K57" s="65">
-        <f t="shared" si="25"/>
-        <v>0.09489005351</v>
+        <f t="shared" si="26"/>
+        <v>0.09589910832</v>
       </c>
       <c r="L57" s="65">
-        <f t="shared" si="25"/>
-        <v>0.0996483074</v>
+        <f t="shared" si="26"/>
+        <v>0.1126105731</v>
       </c>
       <c r="M57" s="65">
-        <f t="shared" si="25"/>
-        <v>0.1046411593</v>
+        <f t="shared" si="26"/>
+        <v>0.1180024754</v>
       </c>
       <c r="N57" s="65">
-        <f t="shared" si="25"/>
-        <v>0.1098802395</v>
+        <f t="shared" si="26"/>
+        <v>0.1236603571</v>
       </c>
       <c r="O57" s="1"/>
       <c r="P57" s="1"/>
@@ -3828,13 +3825,13 @@
       <c r="C59" s="66"/>
       <c r="D59" s="66"/>
       <c r="E59" s="67" t="s">
+        <v>53</v>
+      </c>
+      <c r="F59" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="F59" s="68" t="s">
+      <c r="G59" s="68" t="s">
         <v>55</v>
-      </c>
-      <c r="G59" s="68" t="s">
-        <v>56</v>
       </c>
       <c r="H59" s="69"/>
       <c r="I59" s="70"/>
@@ -3861,19 +3858,19 @@
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
       <c r="C60" s="71" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D60" s="72"/>
       <c r="E60" s="68" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F60" s="73">
         <f>K44/0.07</f>
-        <v>4551959.665</v>
+        <v>4640328.799</v>
       </c>
       <c r="G60" s="74">
-        <f t="array" ref="G60">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+(0.7*F60)})</f>
-        <v>0.1618205601</v>
+        <f t="array" ref="G60">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+1650000+(0.7*(F60-1650000-1989500))})</f>
+        <v>0.1293663886</v>
       </c>
       <c r="H60" s="69"/>
       <c r="I60" s="69"/>
@@ -3901,16 +3898,16 @@
       <c r="B61" s="1"/>
       <c r="C61" s="75"/>
       <c r="D61" s="76"/>
-      <c r="E61" s="68" t="s">
-        <v>59</v>
+      <c r="E61" s="67" t="s">
+        <v>58</v>
       </c>
       <c r="F61" s="73">
-        <f>I44/0.06</f>
-        <v>4823511.75</v>
+        <f>K44/0.065</f>
+        <v>4997277.168</v>
       </c>
       <c r="G61" s="74">
-        <f t="array" ref="G61">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+(0.7*F61)})</f>
-        <v>0.1695799569</v>
+        <f t="array" ref="G61">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+1650000+(0.7*(F61-1650000-1989500))})</f>
+        <v>0.1420913128</v>
       </c>
       <c r="H61" s="69"/>
       <c r="I61" s="69"/>
@@ -3938,16 +3935,16 @@
       <c r="B62" s="1"/>
       <c r="C62" s="75"/>
       <c r="D62" s="76"/>
-      <c r="E62" s="68" t="s">
-        <v>60</v>
+      <c r="E62" s="67" t="s">
+        <v>59</v>
       </c>
       <c r="F62" s="73">
-        <f>K44/0.05</f>
-        <v>6372743.531</v>
+        <f>K44/0.06</f>
+        <v>5413716.932</v>
       </c>
       <c r="G62" s="74">
-        <f t="array" ref="G62">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+(0.7+F62)})</f>
-        <v>0.2621468925</v>
+        <f t="array" ref="G62">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+1650000+(0.7*(F62-1650000-1989500))})</f>
+        <v>0.1558604601</v>
       </c>
       <c r="H62" s="69"/>
       <c r="I62" s="69"/>
@@ -3976,15 +3973,15 @@
       <c r="C63" s="77"/>
       <c r="D63" s="78"/>
       <c r="E63" s="79" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F63" s="73">
-        <f>K44/0.04</f>
-        <v>7965929.414</v>
+        <f>K44/0.055</f>
+        <v>5905873.017</v>
       </c>
       <c r="G63" s="74">
-        <f t="array" ref="G63">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+(0.7*F63)})</f>
-        <v>0.2415566686</v>
+        <f t="array" ref="G63">IRR({D54,E54,F54+F55,G54+G55,H54+H55,I54+I55,J54+J55,K54+K55+1650000+(0.7*(F63-1650000-1989500))})</f>
+        <v>0.170873895</v>
       </c>
       <c r="H63" s="69"/>
       <c r="I63" s="69"/>
@@ -4070,34 +4067,34 @@
       <c r="B66" s="1"/>
       <c r="C66" s="69"/>
       <c r="D66" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E66" s="40" t="str">
-        <f t="shared" ref="E66:K66" si="26">(E30+E32+E36+#REF!+E37+E38+E39+E40+E33)/$D$4</f>
+        <f t="shared" ref="E66:K66" si="27">(E30+E32+E36+#REF!+E37+E38+E39+E40+E33)/$D$4</f>
         <v>#REF!</v>
       </c>
       <c r="F66" s="40" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>#REF!</v>
       </c>
       <c r="G66" s="40" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>#REF!</v>
       </c>
       <c r="H66" s="40" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>#REF!</v>
       </c>
       <c r="I66" s="40" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>#REF!</v>
       </c>
       <c r="J66" s="40" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>#REF!</v>
       </c>
       <c r="K66" s="40" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>#REF!</v>
       </c>
       <c r="L66" s="1"/>
@@ -4122,34 +4119,34 @@
       <c r="B67" s="1"/>
       <c r="C67" s="69"/>
       <c r="D67" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E67" s="40">
-        <f t="shared" ref="E67:K67" si="27">E34/$D$4</f>
+        <f t="shared" ref="E67:K67" si="28">E34/$D$4</f>
         <v>3.441717236</v>
       </c>
       <c r="F67" s="40">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>4.619146816</v>
       </c>
       <c r="G67" s="40">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>4.757721221</v>
       </c>
       <c r="H67" s="40">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>4.900452858</v>
       </c>
       <c r="I67" s="40">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>5.047466443</v>
       </c>
       <c r="J67" s="40">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>5.198890437</v>
       </c>
       <c r="K67" s="40">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>5.35485715</v>
       </c>
       <c r="L67" s="1"/>
@@ -4174,34 +4171,34 @@
       <c r="B68" s="1"/>
       <c r="C68" s="70"/>
       <c r="D68" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E68" s="40">
-        <f t="shared" ref="E68:K68" si="28">E35/$D$4</f>
+        <f t="shared" ref="E68:K68" si="29">E35/$D$4</f>
         <v>1.6</v>
       </c>
       <c r="F68" s="40">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1.648</v>
       </c>
       <c r="G68" s="40">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1.69744</v>
       </c>
       <c r="H68" s="40">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1.7483632</v>
       </c>
       <c r="I68" s="40">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1.800814096</v>
       </c>
       <c r="J68" s="40">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1.854838519</v>
       </c>
       <c r="K68" s="40">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>1.910483674</v>
       </c>
       <c r="L68" s="1"/>
@@ -4257,7 +4254,7 @@
       <c r="B70" s="1"/>
       <c r="C70" s="1"/>
       <c r="D70" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E70" s="1" t="str">
         <f>SUM(E66:E68)</f>
@@ -4268,19 +4265,19 @@
         <v>#REF!</v>
       </c>
       <c r="G70" s="1" t="str">
-        <f t="shared" ref="G70:J70" si="29">SUM(G66:G68)</f>
+        <f t="shared" ref="G70:J70" si="30">SUM(G66:G68)</f>
         <v>#REF!</v>
       </c>
       <c r="H70" s="1" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>#REF!</v>
       </c>
       <c r="I70" s="1" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>#REF!</v>
       </c>
       <c r="J70" s="1" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>#REF!</v>
       </c>
       <c r="K70" s="1"/>
@@ -31014,7 +31011,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="81" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B1" s="81"/>
       <c r="C1" s="81"/>
@@ -31024,7 +31021,7 @@
     </row>
     <row r="2">
       <c r="A2" s="82" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B2" s="82"/>
       <c r="C2" s="82"/>
@@ -31034,7 +31031,7 @@
     </row>
     <row r="3">
       <c r="A3" s="83" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B3" s="83"/>
       <c r="C3" s="83"/>
@@ -31044,57 +31041,57 @@
     </row>
     <row r="5">
       <c r="A5" s="84" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="C5" s="84" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="84" t="s">
+      <c r="D5" s="84" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="84" t="s">
+      <c r="E5" s="84" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="84" t="s">
-        <v>72</v>
-      </c>
       <c r="F5" s="85" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="G5" s="86" t="s">
+      <c r="H5" s="86" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="86" t="s">
+      <c r="I5" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="86" t="s">
+      <c r="J5" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="86" t="s">
+      <c r="K5" s="86" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="86" t="s">
+      <c r="L5" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="86" t="s">
+      <c r="M5" s="86" t="s">
         <v>22</v>
       </c>
-      <c r="M5" s="86" t="s">
+      <c r="N5" s="86" t="s">
         <v>23</v>
       </c>
-      <c r="N5" s="86" t="s">
+      <c r="O5" s="86" t="s">
         <v>24</v>
-      </c>
-      <c r="O5" s="86" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="87" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="87" t="s">
         <v>73</v>
-      </c>
-      <c r="B6" s="87" t="s">
-        <v>74</v>
       </c>
       <c r="C6" s="88">
         <v>952.0</v>
@@ -31110,47 +31107,47 @@
       </c>
       <c r="G6" s="90">
         <f t="shared" ref="G6:G8" si="2">$C$20*C6</f>
-        <v>23324</v>
+        <v>23800</v>
       </c>
       <c r="H6" s="90">
         <f t="shared" ref="H6:O6" si="1">G6*1.05</f>
-        <v>24490.2</v>
+        <v>24990</v>
       </c>
       <c r="I6" s="90">
         <f t="shared" si="1"/>
-        <v>25714.71</v>
+        <v>26239.5</v>
       </c>
       <c r="J6" s="90">
         <f t="shared" si="1"/>
-        <v>27000.4455</v>
+        <v>27551.475</v>
       </c>
       <c r="K6" s="90">
         <f t="shared" si="1"/>
-        <v>28350.46778</v>
+        <v>28929.04875</v>
       </c>
       <c r="L6" s="90">
         <f t="shared" si="1"/>
-        <v>29767.99116</v>
+        <v>30375.50119</v>
       </c>
       <c r="M6" s="90">
         <f t="shared" si="1"/>
-        <v>31256.39072</v>
+        <v>31894.27625</v>
       </c>
       <c r="N6" s="90">
         <f t="shared" si="1"/>
-        <v>32819.21026</v>
+        <v>33488.99006</v>
       </c>
       <c r="O6" s="90">
         <f t="shared" si="1"/>
-        <v>34460.17077</v>
+        <v>35163.43956</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="87" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="87" t="s">
         <v>75</v>
-      </c>
-      <c r="B7" s="87" t="s">
-        <v>76</v>
       </c>
       <c r="C7" s="88">
         <v>750.0</v>
@@ -31166,47 +31163,47 @@
       </c>
       <c r="G7" s="90">
         <f t="shared" si="2"/>
-        <v>18375</v>
+        <v>18750</v>
       </c>
       <c r="H7" s="90">
         <f t="shared" ref="H7:O7" si="3">G7*1.05</f>
-        <v>19293.75</v>
+        <v>19687.5</v>
       </c>
       <c r="I7" s="90">
         <f t="shared" si="3"/>
-        <v>20258.4375</v>
+        <v>20671.875</v>
       </c>
       <c r="J7" s="90">
         <f t="shared" si="3"/>
-        <v>21271.35938</v>
+        <v>21705.46875</v>
       </c>
       <c r="K7" s="90">
         <f t="shared" si="3"/>
-        <v>22334.92734</v>
+        <v>22790.74219</v>
       </c>
       <c r="L7" s="90">
         <f t="shared" si="3"/>
-        <v>23451.67371</v>
+        <v>23930.2793</v>
       </c>
       <c r="M7" s="90">
         <f t="shared" si="3"/>
-        <v>24624.2574</v>
+        <v>25126.79326</v>
       </c>
       <c r="N7" s="90">
         <f t="shared" si="3"/>
-        <v>25855.47027</v>
+        <v>26383.13292</v>
       </c>
       <c r="O7" s="90">
         <f t="shared" si="3"/>
-        <v>27148.24378</v>
+        <v>27702.28957</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="87" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="87" t="s">
         <v>77</v>
-      </c>
-      <c r="B8" s="87" t="s">
-        <v>78</v>
       </c>
       <c r="C8" s="88">
         <v>789.0</v>
@@ -31222,47 +31219,47 @@
       </c>
       <c r="G8" s="90">
         <f t="shared" si="2"/>
-        <v>19330.5</v>
+        <v>19725</v>
       </c>
       <c r="H8" s="90">
         <f t="shared" ref="H8:O8" si="4">G8*1.05</f>
-        <v>20297.025</v>
+        <v>20711.25</v>
       </c>
       <c r="I8" s="90">
         <f t="shared" si="4"/>
-        <v>21311.87625</v>
+        <v>21746.8125</v>
       </c>
       <c r="J8" s="90">
         <f t="shared" si="4"/>
-        <v>22377.47006</v>
+        <v>22834.15313</v>
       </c>
       <c r="K8" s="90">
         <f t="shared" si="4"/>
-        <v>23496.34357</v>
+        <v>23975.86078</v>
       </c>
       <c r="L8" s="90">
         <f t="shared" si="4"/>
-        <v>24671.16074</v>
+        <v>25174.65382</v>
       </c>
       <c r="M8" s="90">
         <f t="shared" si="4"/>
-        <v>25904.71878</v>
+        <v>26433.38651</v>
       </c>
       <c r="N8" s="90">
         <f t="shared" si="4"/>
-        <v>27199.95472</v>
+        <v>27755.05584</v>
       </c>
       <c r="O8" s="90">
         <f t="shared" si="4"/>
-        <v>28559.95246</v>
+        <v>29142.80863</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="87" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="87" t="s">
         <v>79</v>
-      </c>
-      <c r="B9" s="87" t="s">
-        <v>80</v>
       </c>
       <c r="C9" s="88">
         <v>1000.0</v>
@@ -31275,51 +31272,51 @@
       </c>
       <c r="F9" s="89">
         <f>C20*C9</f>
-        <v>24500</v>
+        <v>25000</v>
       </c>
       <c r="G9" s="91">
         <f t="shared" ref="G9:O9" si="5">F9*1.05</f>
-        <v>25725</v>
+        <v>26250</v>
       </c>
       <c r="H9" s="91">
         <f t="shared" si="5"/>
-        <v>27011.25</v>
+        <v>27562.5</v>
       </c>
       <c r="I9" s="91">
         <f t="shared" si="5"/>
-        <v>28361.8125</v>
+        <v>28940.625</v>
       </c>
       <c r="J9" s="91">
         <f t="shared" si="5"/>
-        <v>29779.90313</v>
+        <v>30387.65625</v>
       </c>
       <c r="K9" s="91">
         <f t="shared" si="5"/>
-        <v>31268.89828</v>
+        <v>31907.03906</v>
       </c>
       <c r="L9" s="91">
         <f t="shared" si="5"/>
-        <v>32832.3432</v>
+        <v>33502.39102</v>
       </c>
       <c r="M9" s="91">
         <f t="shared" si="5"/>
-        <v>34473.96036</v>
+        <v>35177.51057</v>
       </c>
       <c r="N9" s="91">
         <f t="shared" si="5"/>
-        <v>36197.65837</v>
+        <v>36936.38609</v>
       </c>
       <c r="O9" s="91">
         <f t="shared" si="5"/>
-        <v>38007.54129</v>
+        <v>38783.2054</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="87" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="87" t="s">
         <v>81</v>
-      </c>
-      <c r="B10" s="87" t="s">
-        <v>82</v>
       </c>
       <c r="C10" s="88">
         <v>3150.0</v>
@@ -31335,47 +31332,47 @@
       </c>
       <c r="G10" s="90">
         <f t="shared" ref="G10:G16" si="7">$C$20*C10</f>
-        <v>77175</v>
+        <v>78750</v>
       </c>
       <c r="H10" s="90">
         <f t="shared" ref="H10:O10" si="6">G10*1.05</f>
-        <v>81033.75</v>
+        <v>82687.5</v>
       </c>
       <c r="I10" s="90">
         <f t="shared" si="6"/>
-        <v>85085.4375</v>
+        <v>86821.875</v>
       </c>
       <c r="J10" s="90">
         <f t="shared" si="6"/>
-        <v>89339.70938</v>
+        <v>91162.96875</v>
       </c>
       <c r="K10" s="90">
         <f t="shared" si="6"/>
-        <v>93806.69484</v>
+        <v>95721.11719</v>
       </c>
       <c r="L10" s="90">
         <f t="shared" si="6"/>
-        <v>98497.02959</v>
+        <v>100507.173</v>
       </c>
       <c r="M10" s="90">
         <f t="shared" si="6"/>
-        <v>103421.8811</v>
+        <v>105532.5317</v>
       </c>
       <c r="N10" s="90">
         <f t="shared" si="6"/>
-        <v>108592.9751</v>
+        <v>110809.1583</v>
       </c>
       <c r="O10" s="90">
         <f t="shared" si="6"/>
-        <v>114022.6239</v>
+        <v>116349.6162</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="87" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="87" t="s">
         <v>83</v>
-      </c>
-      <c r="B11" s="87" t="s">
-        <v>84</v>
       </c>
       <c r="C11" s="88">
         <v>1009.0</v>
@@ -31391,47 +31388,47 @@
       </c>
       <c r="G11" s="90">
         <f t="shared" si="7"/>
-        <v>24720.5</v>
+        <v>25225</v>
       </c>
       <c r="H11" s="90">
         <f t="shared" ref="H11:O11" si="8">G11*1.05</f>
-        <v>25956.525</v>
+        <v>26486.25</v>
       </c>
       <c r="I11" s="90">
         <f t="shared" si="8"/>
-        <v>27254.35125</v>
+        <v>27810.5625</v>
       </c>
       <c r="J11" s="90">
         <f t="shared" si="8"/>
-        <v>28617.06881</v>
+        <v>29201.09063</v>
       </c>
       <c r="K11" s="90">
         <f t="shared" si="8"/>
-        <v>30047.92225</v>
+        <v>30661.14516</v>
       </c>
       <c r="L11" s="90">
         <f t="shared" si="8"/>
-        <v>31550.31837</v>
+        <v>32194.20241</v>
       </c>
       <c r="M11" s="90">
         <f t="shared" si="8"/>
-        <v>33127.83428</v>
+        <v>33803.91253</v>
       </c>
       <c r="N11" s="90">
         <f t="shared" si="8"/>
-        <v>34784.226</v>
+        <v>35494.10816</v>
       </c>
       <c r="O11" s="90">
         <f t="shared" si="8"/>
-        <v>36523.4373</v>
+        <v>37268.81357</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="87" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="87" t="s">
         <v>85</v>
-      </c>
-      <c r="B12" s="87" t="s">
-        <v>86</v>
       </c>
       <c r="C12" s="88">
         <v>1200.0</v>
@@ -31447,47 +31444,47 @@
       </c>
       <c r="G12" s="90">
         <f t="shared" si="7"/>
-        <v>29400</v>
+        <v>30000</v>
       </c>
       <c r="H12" s="90">
         <f t="shared" ref="H12:O12" si="9">G12*1.05</f>
-        <v>30870</v>
+        <v>31500</v>
       </c>
       <c r="I12" s="90">
         <f t="shared" si="9"/>
-        <v>32413.5</v>
+        <v>33075</v>
       </c>
       <c r="J12" s="90">
         <f t="shared" si="9"/>
-        <v>34034.175</v>
+        <v>34728.75</v>
       </c>
       <c r="K12" s="90">
         <f t="shared" si="9"/>
-        <v>35735.88375</v>
+        <v>36465.1875</v>
       </c>
       <c r="L12" s="90">
         <f t="shared" si="9"/>
-        <v>37522.67794</v>
+        <v>38288.44688</v>
       </c>
       <c r="M12" s="90">
         <f t="shared" si="9"/>
-        <v>39398.81183</v>
+        <v>40202.86922</v>
       </c>
       <c r="N12" s="90">
         <f t="shared" si="9"/>
-        <v>41368.75243</v>
+        <v>42213.01268</v>
       </c>
       <c r="O12" s="90">
         <f t="shared" si="9"/>
-        <v>43437.19005</v>
+        <v>44323.66331</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="87" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="87" t="s">
         <v>87</v>
-      </c>
-      <c r="B13" s="87" t="s">
-        <v>88</v>
       </c>
       <c r="C13" s="88">
         <v>550.0</v>
@@ -31503,47 +31500,47 @@
       </c>
       <c r="G13" s="90">
         <f t="shared" si="7"/>
-        <v>13475</v>
+        <v>13750</v>
       </c>
       <c r="H13" s="90">
         <f t="shared" ref="H13:O13" si="10">G13*1.05</f>
-        <v>14148.75</v>
+        <v>14437.5</v>
       </c>
       <c r="I13" s="90">
         <f t="shared" si="10"/>
-        <v>14856.1875</v>
+        <v>15159.375</v>
       </c>
       <c r="J13" s="90">
         <f t="shared" si="10"/>
-        <v>15598.99688</v>
+        <v>15917.34375</v>
       </c>
       <c r="K13" s="90">
         <f t="shared" si="10"/>
-        <v>16378.94672</v>
+        <v>16713.21094</v>
       </c>
       <c r="L13" s="90">
         <f t="shared" si="10"/>
-        <v>17197.89405</v>
+        <v>17548.87148</v>
       </c>
       <c r="M13" s="90">
         <f t="shared" si="10"/>
-        <v>18057.78876</v>
+        <v>18426.31506</v>
       </c>
       <c r="N13" s="90">
         <f t="shared" si="10"/>
-        <v>18960.6782</v>
+        <v>19347.63081</v>
       </c>
       <c r="O13" s="90">
         <f t="shared" si="10"/>
-        <v>19908.71211</v>
+        <v>20315.01235</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="87" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="87" t="s">
         <v>89</v>
-      </c>
-      <c r="B14" s="87" t="s">
-        <v>90</v>
       </c>
       <c r="C14" s="88">
         <v>1041.0</v>
@@ -31559,47 +31556,47 @@
       </c>
       <c r="G14" s="90">
         <f t="shared" si="7"/>
-        <v>25504.5</v>
+        <v>26025</v>
       </c>
       <c r="H14" s="90">
         <f t="shared" ref="H14:O14" si="11">G14*1.05</f>
-        <v>26779.725</v>
+        <v>27326.25</v>
       </c>
       <c r="I14" s="90">
         <f t="shared" si="11"/>
-        <v>28118.71125</v>
+        <v>28692.5625</v>
       </c>
       <c r="J14" s="90">
         <f t="shared" si="11"/>
-        <v>29524.64681</v>
+        <v>30127.19063</v>
       </c>
       <c r="K14" s="90">
         <f t="shared" si="11"/>
-        <v>31000.87915</v>
+        <v>31633.55016</v>
       </c>
       <c r="L14" s="90">
         <f t="shared" si="11"/>
-        <v>32550.92311</v>
+        <v>33215.22766</v>
       </c>
       <c r="M14" s="90">
         <f t="shared" si="11"/>
-        <v>34178.46927</v>
+        <v>34875.98905</v>
       </c>
       <c r="N14" s="90">
         <f t="shared" si="11"/>
-        <v>35887.39273</v>
+        <v>36619.7885</v>
       </c>
       <c r="O14" s="90">
         <f t="shared" si="11"/>
-        <v>37681.76237</v>
+        <v>38450.77792</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="87" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="87" t="s">
         <v>91</v>
-      </c>
-      <c r="B15" s="87" t="s">
-        <v>92</v>
       </c>
       <c r="C15" s="88">
         <v>300.0</v>
@@ -31616,47 +31613,47 @@
       </c>
       <c r="G15" s="90">
         <f t="shared" si="7"/>
-        <v>7350</v>
+        <v>7500</v>
       </c>
       <c r="H15" s="90">
         <f t="shared" ref="H15:O15" si="12">G15*1.05</f>
-        <v>7717.5</v>
+        <v>7875</v>
       </c>
       <c r="I15" s="90">
         <f t="shared" si="12"/>
-        <v>8103.375</v>
+        <v>8268.75</v>
       </c>
       <c r="J15" s="90">
         <f t="shared" si="12"/>
-        <v>8508.54375</v>
+        <v>8682.1875</v>
       </c>
       <c r="K15" s="90">
         <f t="shared" si="12"/>
-        <v>8933.970938</v>
+        <v>9116.296875</v>
       </c>
       <c r="L15" s="90">
         <f t="shared" si="12"/>
-        <v>9380.669484</v>
+        <v>9572.111719</v>
       </c>
       <c r="M15" s="90">
         <f t="shared" si="12"/>
-        <v>9849.702959</v>
+        <v>10050.7173</v>
       </c>
       <c r="N15" s="90">
         <f t="shared" si="12"/>
-        <v>10342.18811</v>
+        <v>10553.25317</v>
       </c>
       <c r="O15" s="90">
         <f t="shared" si="12"/>
-        <v>10859.29751</v>
+        <v>11080.91583</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="87" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="87" t="s">
         <v>93</v>
-      </c>
-      <c r="B16" s="87" t="s">
-        <v>94</v>
       </c>
       <c r="C16" s="88">
         <v>300.0</v>
@@ -31673,44 +31670,44 @@
       </c>
       <c r="G16" s="90">
         <f t="shared" si="7"/>
-        <v>7350</v>
+        <v>7500</v>
       </c>
       <c r="H16" s="90">
         <f t="shared" ref="H16:O16" si="14">G16*1.05</f>
-        <v>7717.5</v>
+        <v>7875</v>
       </c>
       <c r="I16" s="90">
         <f t="shared" si="14"/>
-        <v>8103.375</v>
+        <v>8268.75</v>
       </c>
       <c r="J16" s="90">
         <f t="shared" si="14"/>
-        <v>8508.54375</v>
+        <v>8682.1875</v>
       </c>
       <c r="K16" s="90">
         <f t="shared" si="14"/>
-        <v>8933.970938</v>
+        <v>9116.296875</v>
       </c>
       <c r="L16" s="90">
         <f t="shared" si="14"/>
-        <v>9380.669484</v>
+        <v>9572.111719</v>
       </c>
       <c r="M16" s="90">
         <f t="shared" si="14"/>
-        <v>9849.702959</v>
+        <v>10050.7173</v>
       </c>
       <c r="N16" s="90">
         <f t="shared" si="14"/>
-        <v>10342.18811</v>
+        <v>10553.25317</v>
       </c>
       <c r="O16" s="90">
         <f t="shared" si="14"/>
-        <v>10859.29751</v>
+        <v>11080.91583</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="93" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B17" s="94"/>
       <c r="C17" s="95">
@@ -31724,81 +31721,81 @@
       </c>
       <c r="F17" s="96">
         <f t="shared" si="15"/>
-        <v>265112</v>
+        <v>265612</v>
       </c>
       <c r="G17" s="97">
         <f t="shared" si="15"/>
-        <v>271729.5</v>
+        <v>277275</v>
       </c>
       <c r="H17" s="97">
         <f t="shared" si="15"/>
-        <v>285315.975</v>
+        <v>291138.75</v>
       </c>
       <c r="I17" s="97">
         <f t="shared" si="15"/>
-        <v>299581.7738</v>
+        <v>305695.6875</v>
       </c>
       <c r="J17" s="97">
         <f t="shared" si="15"/>
-        <v>314560.8624</v>
+        <v>320980.4719</v>
       </c>
       <c r="K17" s="97">
         <f t="shared" si="15"/>
-        <v>330288.9056</v>
+        <v>337029.4955</v>
       </c>
       <c r="L17" s="97">
         <f t="shared" si="15"/>
-        <v>346803.3508</v>
+        <v>353880.9702</v>
       </c>
       <c r="M17" s="97">
         <f t="shared" si="15"/>
-        <v>364143.5184</v>
+        <v>371575.0188</v>
       </c>
       <c r="N17" s="97">
         <f t="shared" si="15"/>
-        <v>382350.6943</v>
+        <v>390153.7697</v>
       </c>
       <c r="O17" s="97">
         <f t="shared" si="15"/>
-        <v>401468.229</v>
+        <v>409661.4582</v>
       </c>
     </row>
     <row r="18">
-      <c r="F18" s="98">
-        <f>F17/Proforma!$D$4</f>
-        <v>24.01159315</v>
-      </c>
-      <c r="G18" s="99">
-        <f>G17/Proforma!$D$4</f>
-        <v>24.6109501</v>
-      </c>
-      <c r="H18" s="99">
-        <f>H17/Proforma!$D$4</f>
-        <v>25.8414976</v>
-      </c>
-      <c r="I18" s="99">
-        <f>I17/Proforma!$D$4</f>
-        <v>27.13357248</v>
-      </c>
-      <c r="J18" s="99">
-        <f>J17/Proforma!$D$4</f>
-        <v>28.4902511</v>
-      </c>
-      <c r="K18" s="99">
-        <f>K17/Proforma!$D$4</f>
-        <v>29.91476366</v>
-      </c>
-      <c r="L18" s="99">
-        <f>L17/Proforma!$D$4</f>
-        <v>31.41050184</v>
+      <c r="F18" s="98" t="str">
+        <f t="shared" ref="F18:L18" si="16">F17/Proforma!$D$4</f>
+        <v>#REF!</v>
+      </c>
+      <c r="G18" s="99" t="str">
+        <f t="shared" si="16"/>
+        <v>#REF!</v>
+      </c>
+      <c r="H18" s="99" t="str">
+        <f t="shared" si="16"/>
+        <v>#REF!</v>
+      </c>
+      <c r="I18" s="99" t="str">
+        <f t="shared" si="16"/>
+        <v>#REF!</v>
+      </c>
+      <c r="J18" s="99" t="str">
+        <f t="shared" si="16"/>
+        <v>#REF!</v>
+      </c>
+      <c r="K18" s="99" t="str">
+        <f t="shared" si="16"/>
+        <v>#REF!</v>
+      </c>
+      <c r="L18" s="99" t="str">
+        <f t="shared" si="16"/>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="100" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C20" s="101">
-        <v>24.5</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -32809,57 +32806,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="81" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="82" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="83" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="102" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="102" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="102" t="s">
+      <c r="C5" s="102" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="102" t="s">
+      <c r="D5" s="102" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="102" t="s">
+      <c r="E5" s="102" t="s">
+        <v>96</v>
+      </c>
+      <c r="F5" s="102" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="102" t="s">
+      <c r="G5" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="F5" s="102" t="s">
-        <v>72</v>
-      </c>
-      <c r="G5" s="102" t="s">
+      <c r="H5" s="102" t="s">
         <v>98</v>
       </c>
-      <c r="H5" s="102" t="s">
+      <c r="I5" s="102" t="s">
         <v>99</v>
       </c>
-      <c r="I5" s="102" t="s">
+      <c r="J5" s="102" t="s">
         <v>100</v>
-      </c>
-      <c r="J5" s="102" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="87" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="87" t="s">
         <v>73</v>
-      </c>
-      <c r="B6" s="87" t="s">
-        <v>74</v>
       </c>
       <c r="C6" s="87">
         <v>952.0</v>
@@ -32875,19 +32872,19 @@
       </c>
       <c r="G6" s="87"/>
       <c r="H6" s="87" t="s">
+        <v>101</v>
+      </c>
+      <c r="I6" s="87" t="s">
         <v>102</v>
-      </c>
-      <c r="I6" s="87" t="s">
-        <v>103</v>
       </c>
       <c r="J6" s="87"/>
     </row>
     <row r="7">
       <c r="A7" s="87" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="87" t="s">
         <v>75</v>
-      </c>
-      <c r="B7" s="87" t="s">
-        <v>76</v>
       </c>
       <c r="C7" s="87">
         <v>750.0</v>
@@ -32903,19 +32900,19 @@
       </c>
       <c r="G7" s="87"/>
       <c r="H7" s="87" t="s">
+        <v>103</v>
+      </c>
+      <c r="I7" s="87" t="s">
         <v>104</v>
-      </c>
-      <c r="I7" s="87" t="s">
-        <v>105</v>
       </c>
       <c r="J7" s="87"/>
     </row>
     <row r="8">
       <c r="A8" s="87" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="87" t="s">
         <v>77</v>
-      </c>
-      <c r="B8" s="87" t="s">
-        <v>78</v>
       </c>
       <c r="C8" s="87">
         <v>789.0</v>
@@ -32931,19 +32928,19 @@
       </c>
       <c r="G8" s="87"/>
       <c r="H8" s="87" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I8" s="87" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J8" s="87"/>
     </row>
     <row r="9">
       <c r="A9" s="87" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="87" t="s">
         <v>79</v>
-      </c>
-      <c r="B9" s="87" t="s">
-        <v>80</v>
       </c>
       <c r="C9" s="87">
         <v>1000.0</v>
@@ -32958,22 +32955,22 @@
         <v>500.0</v>
       </c>
       <c r="G9" s="87" t="s">
+        <v>106</v>
+      </c>
+      <c r="H9" s="87" t="s">
         <v>107</v>
       </c>
-      <c r="H9" s="87" t="s">
+      <c r="I9" s="87" t="s">
         <v>108</v>
-      </c>
-      <c r="I9" s="87" t="s">
-        <v>109</v>
       </c>
       <c r="J9" s="87"/>
     </row>
     <row r="10">
       <c r="A10" s="87" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="87" t="s">
         <v>81</v>
-      </c>
-      <c r="B10" s="87" t="s">
-        <v>82</v>
       </c>
       <c r="C10" s="87">
         <v>3150.0</v>
@@ -32988,24 +32985,24 @@
         <v>7569.17</v>
       </c>
       <c r="G10" s="87" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H10" s="87" t="s">
+        <v>109</v>
+      </c>
+      <c r="I10" s="87" t="s">
         <v>110</v>
       </c>
-      <c r="I10" s="87" t="s">
+      <c r="J10" s="87" t="s">
         <v>111</v>
-      </c>
-      <c r="J10" s="87" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="87" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="87" t="s">
         <v>83</v>
-      </c>
-      <c r="B11" s="87" t="s">
-        <v>84</v>
       </c>
       <c r="C11" s="87">
         <v>1009.0</v>
@@ -33020,24 +33017,24 @@
         <v>1836.11</v>
       </c>
       <c r="G11" s="87" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H11" s="87" t="s">
+        <v>112</v>
+      </c>
+      <c r="I11" s="87" t="s">
         <v>113</v>
       </c>
-      <c r="I11" s="87" t="s">
-        <v>114</v>
-      </c>
       <c r="J11" s="87" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="87" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="87" t="s">
         <v>85</v>
-      </c>
-      <c r="B12" s="87" t="s">
-        <v>86</v>
       </c>
       <c r="C12" s="87">
         <v>1200.0</v>
@@ -33052,22 +33049,22 @@
         <v>2669.0</v>
       </c>
       <c r="G12" s="87" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H12" s="87" t="s">
+        <v>114</v>
+      </c>
+      <c r="I12" s="87" t="s">
         <v>115</v>
-      </c>
-      <c r="I12" s="87" t="s">
-        <v>116</v>
       </c>
       <c r="J12" s="87"/>
     </row>
     <row r="13">
       <c r="A13" s="87" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="87" t="s">
         <v>87</v>
-      </c>
-      <c r="B13" s="87" t="s">
-        <v>88</v>
       </c>
       <c r="C13" s="87">
         <v>550.0</v>
@@ -33082,22 +33079,22 @@
         <v>1051.88</v>
       </c>
       <c r="G13" s="87" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H13" s="87" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="I13" s="87" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J13" s="87"/>
     </row>
     <row r="14">
       <c r="A14" s="87" t="s">
+        <v>88</v>
+      </c>
+      <c r="B14" s="87" t="s">
         <v>89</v>
-      </c>
-      <c r="B14" s="87" t="s">
-        <v>90</v>
       </c>
       <c r="C14" s="87">
         <v>1041.0</v>
@@ -33113,19 +33110,19 @@
       </c>
       <c r="G14" s="87"/>
       <c r="H14" s="87" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I14" s="87" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J14" s="87"/>
     </row>
     <row r="15">
       <c r="A15" s="87" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="87" t="s">
         <v>91</v>
-      </c>
-      <c r="B15" s="87" t="s">
-        <v>92</v>
       </c>
       <c r="C15" s="87">
         <v>300.0</v>
@@ -33140,10 +33137,10 @@
     </row>
     <row r="16">
       <c r="A16" s="87" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="87" t="s">
         <v>93</v>
-      </c>
-      <c r="B16" s="87" t="s">
-        <v>94</v>
       </c>
       <c r="C16" s="87">
         <v>300.0</v>
@@ -33158,7 +33155,7 @@
     </row>
     <row r="17">
       <c r="A17" s="93" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B17" s="94"/>
       <c r="C17" s="95">

</xml_diff>